<commit_message>
removed fixtures for w/c 22nd feb
</commit_message>
<xml_diff>
--- a/in/MRFC-FIXTURES-2024-25.xlsx
+++ b/in/MRFC-FIXTURES-2024-25.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10209"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nickgreen/workspace/code/morleyrfc/morleyrfc-fixtures/in/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68E813FC-F318-794E-94B1-AB327B1992F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85E3AD97-1501-8A47-B0BC-75EE1C947C86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1860" yWindow="760" windowWidth="15420" windowHeight="16440" tabRatio="482" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="161">
   <si>
     <t>Date</t>
   </si>
@@ -2476,16 +2476,10 @@
         <f t="shared" si="1"/>
         <v>45710</v>
       </c>
-      <c r="B32" s="67" t="s">
-        <v>128</v>
-      </c>
+      <c r="B32" s="67"/>
       <c r="C32" s="61"/>
-      <c r="D32" s="72" t="s">
-        <v>131</v>
-      </c>
-      <c r="E32" s="61" t="s">
-        <v>32</v>
-      </c>
+      <c r="D32" s="72"/>
+      <c r="E32" s="61"/>
       <c r="F32" s="5"/>
       <c r="G32" s="36"/>
       <c r="H32" s="38"/>

</xml_diff>

<commit_message>
added latest cup game
</commit_message>
<xml_diff>
--- a/in/MRFC-FIXTURES-2024-25.xlsx
+++ b/in/MRFC-FIXTURES-2024-25.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10402"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nickgreen/workspace/code/morleyrfc/morleyrfc-fixtures/in/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85E3AD97-1501-8A47-B0BC-75EE1C947C86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A12551A-EDF9-564C-BC7D-4BA727D67B2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1860" yWindow="760" windowWidth="15420" windowHeight="16440" tabRatio="482" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="162">
   <si>
     <t>Date</t>
   </si>
@@ -525,6 +525,9 @@
   </si>
   <si>
     <t>Wetherby (PJ Cup)</t>
+  </si>
+  <si>
+    <t>Old Brodleians (PJ Cup)</t>
   </si>
 </sst>
 </file>
@@ -2686,9 +2689,11 @@
         <v>45773</v>
       </c>
       <c r="B41" s="67" t="s">
-        <v>129</v>
-      </c>
-      <c r="C41" s="61"/>
+        <v>161</v>
+      </c>
+      <c r="C41" s="61" t="s">
+        <v>31</v>
+      </c>
       <c r="D41" s="72"/>
       <c r="E41" s="61"/>
       <c r="F41" s="4"/>

</xml_diff>

<commit_message>
updated to finish the season
</commit_message>
<xml_diff>
--- a/in/MRFC-FIXTURES-2024-25.xlsx
+++ b/in/MRFC-FIXTURES-2024-25.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10402"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nickgreen/workspace/code/morleyrfc/morleyrfc-fixtures/in/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A12551A-EDF9-564C-BC7D-4BA727D67B2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7643C90-94FF-604A-9128-1348403D7D8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1860" yWindow="760" windowWidth="15420" windowHeight="16440" tabRatio="482" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,9 +19,9 @@
     <sheet name="YC" sheetId="3" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Fixtures!$A$3:$L$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Fixtures!$A$3:$L$46</definedName>
     <definedName name="Data">YC!#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Fixtures!$A$1:$L$46</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Fixtures!$A$1:$L$44</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <fileRecoveryPr autoRecover="0"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="162">
   <si>
     <t>Date</t>
   </si>
@@ -431,9 +431,6 @@
     <t>TBC</t>
   </si>
   <si>
-    <t>PJ Cup</t>
-  </si>
-  <si>
     <t>Moortown 2</t>
   </si>
   <si>
@@ -528,6 +525,9 @@
   </si>
   <si>
     <t>Old Brodleians (PJ Cup)</t>
+  </si>
+  <si>
+    <t>West Bridgeford (PJ Cup)</t>
   </si>
 </sst>
 </file>
@@ -719,7 +719,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="34">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -885,21 +885,6 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -1053,34 +1038,6 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -1093,19 +1050,6 @@
         <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -1170,7 +1114,7 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="102">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1205,7 +1149,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1218,62 +1162,62 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1281,63 +1225,44 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="16" fontId="4" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1348,22 +1273,19 @@
     <xf numFmtId="16" fontId="4" fillId="6" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="16" fontId="4" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1371,32 +1293,32 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1714,7 +1636,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O115"/>
+  <dimension ref="A1:O113"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.5" style="1" customWidth="1"/>
@@ -1737,36 +1659,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="99" t="s">
-        <v>145</v>
-      </c>
-      <c r="B1" s="100"/>
-      <c r="C1" s="100"/>
-      <c r="D1" s="100"/>
-      <c r="E1" s="100"/>
-      <c r="F1" s="100"/>
-      <c r="G1" s="100"/>
-      <c r="H1" s="100"/>
-      <c r="I1" s="100"/>
-      <c r="J1" s="100"/>
-      <c r="K1" s="100"/>
-      <c r="L1" s="101"/>
+      <c r="A1" s="89" t="s">
+        <v>144</v>
+      </c>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="91"/>
       <c r="N1"/>
       <c r="O1"/>
     </row>
     <row r="2" spans="1:15" ht="5.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58"/>
-      <c r="B2" s="59"/>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="59"/>
-      <c r="F2" s="59"/>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="59"/>
-      <c r="L2" s="82"/>
+      <c r="A2" s="53"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="54"/>
+      <c r="J2" s="54"/>
+      <c r="K2" s="54"/>
+      <c r="L2" s="72"/>
     </row>
     <row r="3" spans="1:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -1775,28 +1697,28 @@
       <c r="B3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="90" t="s">
+      <c r="C3" s="80" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="91" t="s">
+      <c r="D3" s="81" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="90" t="s">
+      <c r="E3" s="80" t="s">
         <v>26</v>
       </c>
-      <c r="F3" s="92"/>
-      <c r="G3" s="93" t="s">
+      <c r="F3" s="82"/>
+      <c r="G3" s="83" t="s">
         <v>26</v>
       </c>
-      <c r="H3" s="94" t="s">
+      <c r="H3" s="84" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="95"/>
-      <c r="J3" s="96" t="s">
+      <c r="I3" s="85"/>
+      <c r="J3" s="86" t="s">
         <v>2</v>
       </c>
-      <c r="K3" s="96"/>
-      <c r="L3" s="97" t="s">
+      <c r="K3" s="86"/>
+      <c r="L3" s="87" t="s">
         <v>10</v>
       </c>
       <c r="O3"/>
@@ -1805,36 +1727,36 @@
       <c r="A4" s="3">
         <v>45514</v>
       </c>
-      <c r="B4" s="83" t="s">
+      <c r="B4" s="73" t="s">
         <v>124</v>
       </c>
-      <c r="C4" s="84" t="s">
+      <c r="C4" s="74" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="83"/>
-      <c r="E4" s="85"/>
-      <c r="F4" s="86"/>
-      <c r="G4" s="87"/>
-      <c r="H4" s="87"/>
-      <c r="I4" s="87"/>
-      <c r="J4" s="88"/>
-      <c r="K4" s="87"/>
-      <c r="L4" s="89" t="s">
+      <c r="D4" s="73"/>
+      <c r="E4" s="75"/>
+      <c r="F4" s="76"/>
+      <c r="G4" s="77"/>
+      <c r="H4" s="77"/>
+      <c r="I4" s="77"/>
+      <c r="J4" s="78"/>
+      <c r="K4" s="77"/>
+      <c r="L4" s="79" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A5" s="78">
+      <c r="A5" s="69">
         <v>45521</v>
       </c>
-      <c r="B5" s="70" t="s">
+      <c r="B5" s="64" t="s">
         <v>123</v>
       </c>
-      <c r="C5" s="75" t="s">
+      <c r="C5" s="68" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="70"/>
-      <c r="E5" s="60"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="55"/>
       <c r="F5" s="4"/>
       <c r="G5" s="34"/>
       <c r="H5" s="34"/>
@@ -1846,35 +1768,35 @@
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A6" s="78">
+      <c r="A6" s="69">
         <v>45526</v>
       </c>
-      <c r="B6" s="70" t="s">
-        <v>144</v>
-      </c>
-      <c r="C6" s="75" t="s">
+      <c r="B6" s="64" t="s">
+        <v>143</v>
+      </c>
+      <c r="C6" s="68" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="70"/>
-      <c r="E6" s="60"/>
+      <c r="D6" s="64"/>
+      <c r="E6" s="55"/>
       <c r="F6" s="4"/>
       <c r="G6" s="34"/>
       <c r="H6" s="34"/>
       <c r="I6" s="34"/>
       <c r="J6" s="33"/>
       <c r="K6" s="34"/>
-      <c r="L6" s="98" t="s">
-        <v>155</v>
+      <c r="L6" s="88" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="7" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="79">
+      <c r="A7" s="70">
         <v>45536</v>
       </c>
-      <c r="B7" s="70"/>
-      <c r="C7" s="75"/>
-      <c r="D7" s="70"/>
-      <c r="E7" s="60"/>
+      <c r="B7" s="64"/>
+      <c r="C7" s="68"/>
+      <c r="D7" s="64"/>
+      <c r="E7" s="55"/>
       <c r="F7" s="4"/>
       <c r="G7" s="34"/>
       <c r="H7" s="34"/>
@@ -1884,19 +1806,19 @@
       <c r="L7" s="47"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A8" s="78">
+      <c r="A8" s="69">
         <v>45542</v>
       </c>
-      <c r="B8" s="67" t="s">
+      <c r="B8" s="62" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="61" t="s">
+      <c r="C8" s="56" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="71" t="s">
-        <v>131</v>
-      </c>
-      <c r="E8" s="61" t="s">
+      <c r="D8" s="65" t="s">
+        <v>130</v>
+      </c>
+      <c r="E8" s="56" t="s">
         <v>31</v>
       </c>
       <c r="F8" s="6"/>
@@ -1908,20 +1830,20 @@
       <c r="L8" s="48"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A9" s="78">
+      <c r="A9" s="69">
         <f>+A8+7</f>
         <v>45549</v>
       </c>
-      <c r="B9" s="67" t="s">
+      <c r="B9" s="62" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="61" t="s">
+      <c r="C9" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="71" t="s">
-        <v>132</v>
-      </c>
-      <c r="E9" s="62" t="s">
+      <c r="D9" s="65" t="s">
+        <v>131</v>
+      </c>
+      <c r="E9" s="57" t="s">
         <v>32</v>
       </c>
       <c r="F9" s="6"/>
@@ -1933,20 +1855,20 @@
       <c r="L9" s="49"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A10" s="78">
+      <c r="A10" s="69">
         <f t="shared" ref="A10:A22" si="0">+A9+7</f>
         <v>45556</v>
       </c>
-      <c r="B10" s="67" t="s">
+      <c r="B10" s="62" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="61" t="s">
+      <c r="C10" s="56" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="70" t="s">
+      <c r="D10" s="64" t="s">
         <v>110</v>
       </c>
-      <c r="E10" s="61" t="s">
+      <c r="E10" s="56" t="s">
         <v>31</v>
       </c>
       <c r="F10" s="4"/>
@@ -1958,20 +1880,20 @@
       <c r="L10" s="50"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A11" s="78">
+      <c r="A11" s="69">
         <f t="shared" si="0"/>
         <v>45563</v>
       </c>
-      <c r="B11" s="67" t="s">
+      <c r="B11" s="62" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="61" t="s">
+      <c r="C11" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="70" t="s">
+      <c r="D11" s="64" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="62" t="s">
+      <c r="E11" s="57" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="4"/>
@@ -1983,18 +1905,18 @@
       <c r="L11" s="50"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A12" s="78">
+      <c r="A12" s="69">
         <f t="shared" si="0"/>
         <v>45570</v>
       </c>
-      <c r="B12" s="67" t="s">
+      <c r="B12" s="62" t="s">
+        <v>141</v>
+      </c>
+      <c r="C12" s="56" t="s">
         <v>142</v>
       </c>
-      <c r="C12" s="61" t="s">
-        <v>143</v>
-      </c>
-      <c r="D12" s="70"/>
-      <c r="E12" s="63"/>
+      <c r="D12" s="64"/>
+      <c r="E12" s="58"/>
       <c r="F12" s="4"/>
       <c r="G12" s="40"/>
       <c r="H12" s="40"/>
@@ -2004,20 +1926,20 @@
       <c r="L12" s="50"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A13" s="78">
+      <c r="A13" s="69">
         <f t="shared" si="0"/>
         <v>45577</v>
       </c>
-      <c r="B13" s="67" t="s">
+      <c r="B13" s="62" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="61" t="s">
+      <c r="C13" s="56" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="72" t="s">
+      <c r="D13" s="66" t="s">
         <v>42</v>
       </c>
-      <c r="E13" s="64" t="s">
+      <c r="E13" s="59" t="s">
         <v>27</v>
       </c>
       <c r="F13" s="4"/>
@@ -2029,20 +1951,20 @@
       <c r="L13" s="50"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A14" s="78">
+      <c r="A14" s="69">
         <f t="shared" si="0"/>
         <v>45584</v>
       </c>
-      <c r="B14" s="67" t="s">
-        <v>157</v>
-      </c>
-      <c r="C14" s="61" t="s">
+      <c r="B14" s="62" t="s">
+        <v>156</v>
+      </c>
+      <c r="C14" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="D14" s="72" t="s">
+      <c r="D14" s="66" t="s">
         <v>40</v>
       </c>
-      <c r="E14" s="64" t="s">
+      <c r="E14" s="59" t="s">
         <v>29</v>
       </c>
       <c r="F14" s="4"/>
@@ -2055,20 +1977,20 @@
       <c r="O14"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A15" s="78">
+      <c r="A15" s="69">
         <f t="shared" si="0"/>
         <v>45591</v>
       </c>
-      <c r="B15" s="67" t="s">
+      <c r="B15" s="62" t="s">
         <v>35</v>
       </c>
-      <c r="C15" s="61" t="s">
+      <c r="C15" s="56" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="70" t="s">
+      <c r="D15" s="64" t="s">
         <v>14</v>
       </c>
-      <c r="E15" s="62" t="s">
+      <c r="E15" s="57" t="s">
         <v>27</v>
       </c>
       <c r="F15" s="4"/>
@@ -2080,16 +2002,16 @@
       <c r="L15" s="50"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A16" s="78">
+      <c r="A16" s="69">
         <f t="shared" si="0"/>
         <v>45598</v>
       </c>
-      <c r="B16" s="67" t="s">
+      <c r="B16" s="62" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="61"/>
-      <c r="D16" s="70"/>
-      <c r="E16" s="65"/>
+      <c r="C16" s="56"/>
+      <c r="D16" s="64"/>
+      <c r="E16" s="60"/>
       <c r="F16" s="4"/>
       <c r="G16" s="40"/>
       <c r="H16" s="40"/>
@@ -2097,24 +2019,24 @@
       <c r="J16" s="33"/>
       <c r="K16" s="34"/>
       <c r="L16" s="50" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A17" s="78">
+      <c r="A17" s="69">
         <f t="shared" si="0"/>
         <v>45605</v>
       </c>
-      <c r="B17" s="67" t="s">
+      <c r="B17" s="62" t="s">
         <v>39</v>
       </c>
-      <c r="C17" s="61" t="s">
+      <c r="C17" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="D17" s="70" t="s">
+      <c r="D17" s="64" t="s">
         <v>33</v>
       </c>
-      <c r="E17" s="61" t="s">
+      <c r="E17" s="56" t="s">
         <v>27</v>
       </c>
       <c r="F17" s="4"/>
@@ -2124,24 +2046,24 @@
       <c r="J17" s="33"/>
       <c r="K17" s="34"/>
       <c r="L17" s="50" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A18" s="78">
+      <c r="A18" s="69">
         <f t="shared" si="0"/>
         <v>45612</v>
       </c>
-      <c r="B18" s="67" t="s">
+      <c r="B18" s="62" t="s">
+        <v>157</v>
+      </c>
+      <c r="C18" s="56" t="s">
+        <v>29</v>
+      </c>
+      <c r="D18" s="64" t="s">
         <v>158</v>
       </c>
-      <c r="C18" s="61" t="s">
-        <v>29</v>
-      </c>
-      <c r="D18" s="70" t="s">
-        <v>159</v>
-      </c>
-      <c r="E18" s="62" t="s">
+      <c r="E18" s="57" t="s">
         <v>32</v>
       </c>
       <c r="F18" s="4"/>
@@ -2151,23 +2073,23 @@
       <c r="J18" s="33"/>
       <c r="K18" s="34"/>
       <c r="L18" s="50" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="N18" s="8"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A19" s="78">
+      <c r="A19" s="69">
         <f t="shared" si="0"/>
         <v>45619</v>
       </c>
-      <c r="B19" s="67" t="s">
+      <c r="B19" s="62" t="s">
+        <v>141</v>
+      </c>
+      <c r="C19" s="56" t="s">
         <v>142</v>
       </c>
-      <c r="C19" s="61" t="s">
-        <v>143</v>
-      </c>
-      <c r="D19" s="70"/>
-      <c r="E19" s="66"/>
+      <c r="D19" s="64"/>
+      <c r="E19" s="61"/>
       <c r="F19" s="4"/>
       <c r="G19" s="40"/>
       <c r="H19" s="35"/>
@@ -2175,25 +2097,25 @@
       <c r="J19" s="33"/>
       <c r="K19" s="34"/>
       <c r="L19" s="50" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N19" s="8"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A20" s="78">
+      <c r="A20" s="69">
         <f t="shared" si="0"/>
         <v>45626</v>
       </c>
-      <c r="B20" s="67" t="s">
+      <c r="B20" s="62" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="61" t="s">
+      <c r="C20" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="D20" s="70" t="s">
-        <v>130</v>
-      </c>
-      <c r="E20" s="62" t="s">
+      <c r="D20" s="64" t="s">
+        <v>129</v>
+      </c>
+      <c r="E20" s="57" t="s">
         <v>29</v>
       </c>
       <c r="F20" s="4"/>
@@ -2206,20 +2128,20 @@
       <c r="N20" s="9"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A21" s="78">
+      <c r="A21" s="69">
         <f t="shared" si="0"/>
         <v>45633</v>
       </c>
-      <c r="B21" s="67" t="s">
+      <c r="B21" s="62" t="s">
         <v>13</v>
       </c>
-      <c r="C21" s="61" t="s">
+      <c r="C21" s="56" t="s">
         <v>29</v>
       </c>
-      <c r="D21" s="70" t="s">
+      <c r="D21" s="64" t="s">
         <v>25</v>
       </c>
-      <c r="E21" s="62" t="s">
+      <c r="E21" s="57" t="s">
         <v>27</v>
       </c>
       <c r="F21" s="6"/>
@@ -2231,20 +2153,20 @@
       <c r="L21" s="50"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A22" s="78">
+      <c r="A22" s="69">
         <f t="shared" si="0"/>
         <v>45640</v>
       </c>
-      <c r="B22" s="67" t="s">
+      <c r="B22" s="62" t="s">
         <v>28</v>
       </c>
-      <c r="C22" s="61" t="s">
+      <c r="C22" s="56" t="s">
         <v>29</v>
       </c>
-      <c r="D22" s="71" t="s">
-        <v>132</v>
-      </c>
-      <c r="E22" s="67" t="s">
+      <c r="D22" s="65" t="s">
+        <v>131</v>
+      </c>
+      <c r="E22" s="62" t="s">
         <v>31</v>
       </c>
       <c r="F22" s="4"/>
@@ -2256,18 +2178,18 @@
       <c r="L22" s="50"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A23" s="78">
+      <c r="A23" s="69">
         <f>+A22+7</f>
         <v>45647</v>
       </c>
-      <c r="B23" s="67" t="s">
+      <c r="B23" s="62" t="s">
         <v>37</v>
       </c>
-      <c r="C23" s="61" t="s">
+      <c r="C23" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="D23" s="72"/>
-      <c r="E23" s="68"/>
+      <c r="D23" s="66"/>
+      <c r="E23" s="63"/>
       <c r="F23" s="5"/>
       <c r="G23" s="41"/>
       <c r="H23" s="41"/>
@@ -2277,16 +2199,16 @@
       <c r="L23" s="50"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A24" s="80">
+      <c r="A24" s="71">
         <f>+A23+7</f>
         <v>45654</v>
       </c>
-      <c r="B24" s="67" t="s">
+      <c r="B24" s="62" t="s">
         <v>30</v>
       </c>
-      <c r="C24" s="61"/>
-      <c r="D24" s="72"/>
-      <c r="E24" s="64"/>
+      <c r="C24" s="56"/>
+      <c r="D24" s="66"/>
+      <c r="E24" s="59"/>
       <c r="F24" s="5"/>
       <c r="G24" s="41"/>
       <c r="H24" s="41"/>
@@ -2298,20 +2220,20 @@
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A25" s="78">
+      <c r="A25" s="69">
         <f t="shared" ref="A25:A37" si="1">+A24+7</f>
         <v>45661</v>
       </c>
-      <c r="B25" s="67" t="s">
+      <c r="B25" s="62" t="s">
         <v>11</v>
       </c>
-      <c r="C25" s="61" t="s">
+      <c r="C25" s="56" t="s">
         <v>29</v>
       </c>
-      <c r="D25" s="72" t="s">
+      <c r="D25" s="66" t="s">
         <v>15</v>
       </c>
-      <c r="E25" s="64" t="s">
+      <c r="E25" s="59" t="s">
         <v>27</v>
       </c>
       <c r="F25" s="5"/>
@@ -2323,23 +2245,23 @@
       <c r="L25" s="50"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A26" s="78">
+      <c r="A26" s="69">
         <f t="shared" si="1"/>
         <v>45668</v>
       </c>
-      <c r="B26" s="67" t="s">
+      <c r="B26" s="62" t="s">
         <v>38</v>
       </c>
-      <c r="C26" s="61" t="s">
+      <c r="C26" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="D26" s="67" t="s">
+      <c r="D26" s="62" t="s">
         <v>42</v>
       </c>
-      <c r="E26" s="67" t="s">
+      <c r="E26" s="62" t="s">
         <v>29</v>
       </c>
-      <c r="F26" s="56"/>
+      <c r="F26" s="52"/>
       <c r="G26" s="35"/>
       <c r="H26" s="39"/>
       <c r="I26" s="38"/>
@@ -2348,20 +2270,20 @@
       <c r="L26" s="50"/>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A27" s="78">
+      <c r="A27" s="69">
         <f t="shared" si="1"/>
         <v>45675</v>
       </c>
-      <c r="B27" s="67" t="s">
-        <v>157</v>
-      </c>
-      <c r="C27" s="61" t="s">
+      <c r="B27" s="62" t="s">
+        <v>156</v>
+      </c>
+      <c r="C27" s="56" t="s">
         <v>29</v>
       </c>
-      <c r="D27" s="70" t="s">
+      <c r="D27" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="E27" s="61" t="s">
+      <c r="E27" s="56" t="s">
         <v>27</v>
       </c>
       <c r="F27" s="4"/>
@@ -2373,18 +2295,18 @@
       <c r="L27" s="50"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A28" s="78">
+      <c r="A28" s="69">
         <f t="shared" si="1"/>
         <v>45682</v>
       </c>
-      <c r="B28" s="67" t="s">
+      <c r="B28" s="62" t="s">
         <v>128</v>
       </c>
-      <c r="C28" s="61"/>
-      <c r="D28" s="70" t="s">
+      <c r="C28" s="56"/>
+      <c r="D28" s="64" t="s">
         <v>33</v>
       </c>
-      <c r="E28" s="61" t="s">
+      <c r="E28" s="56" t="s">
         <v>29</v>
       </c>
       <c r="F28" s="4"/>
@@ -2396,20 +2318,20 @@
       <c r="L28" s="50"/>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A29" s="78">
+      <c r="A29" s="69">
         <f t="shared" si="1"/>
         <v>45689</v>
       </c>
-      <c r="B29" s="67" t="s">
+      <c r="B29" s="62" t="s">
         <v>35</v>
       </c>
-      <c r="C29" s="61" t="s">
+      <c r="C29" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="D29" s="70" t="s">
+      <c r="D29" s="64" t="s">
         <v>14</v>
       </c>
-      <c r="E29" s="61" t="s">
+      <c r="E29" s="56" t="s">
         <v>29</v>
       </c>
       <c r="F29" s="4"/>
@@ -2419,24 +2341,24 @@
       <c r="J29" s="33"/>
       <c r="K29" s="34"/>
       <c r="L29" s="50" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A30" s="78">
+      <c r="A30" s="69">
         <f t="shared" si="1"/>
         <v>45696</v>
       </c>
-      <c r="B30" s="67" t="s">
+      <c r="B30" s="62" t="s">
         <v>38</v>
       </c>
-      <c r="C30" s="61" t="s">
+      <c r="C30" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="D30" s="70" t="s">
+      <c r="D30" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="E30" s="64" t="s">
+      <c r="E30" s="59" t="s">
         <v>27</v>
       </c>
       <c r="F30" s="5"/>
@@ -2446,24 +2368,24 @@
       <c r="J30" s="33"/>
       <c r="K30" s="34"/>
       <c r="L30" s="50" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A31" s="78">
+      <c r="A31" s="69">
         <f t="shared" si="1"/>
         <v>45703</v>
       </c>
-      <c r="B31" s="67" t="s">
+      <c r="B31" s="62" t="s">
         <v>39</v>
       </c>
-      <c r="C31" s="61" t="s">
+      <c r="C31" s="56" t="s">
         <v>29</v>
       </c>
-      <c r="D31" s="73" t="s">
+      <c r="D31" s="67" t="s">
         <v>21</v>
       </c>
-      <c r="E31" s="61" t="s">
+      <c r="E31" s="56" t="s">
         <v>27</v>
       </c>
       <c r="F31" s="4"/>
@@ -2475,14 +2397,14 @@
       <c r="L31" s="50"/>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A32" s="78">
+      <c r="A32" s="69">
         <f t="shared" si="1"/>
         <v>45710</v>
       </c>
-      <c r="B32" s="67"/>
-      <c r="C32" s="61"/>
-      <c r="D32" s="72"/>
-      <c r="E32" s="61"/>
+      <c r="B32" s="62"/>
+      <c r="C32" s="56"/>
+      <c r="D32" s="66"/>
+      <c r="E32" s="56"/>
       <c r="F32" s="5"/>
       <c r="G32" s="36"/>
       <c r="H32" s="38"/>
@@ -2490,25 +2412,25 @@
       <c r="J32" s="33"/>
       <c r="K32" s="34"/>
       <c r="L32" s="50" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="O32"/>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A33" s="78">
+      <c r="A33" s="69">
         <f t="shared" si="1"/>
         <v>45717</v>
       </c>
-      <c r="B33" s="67" t="s">
+      <c r="B33" s="62" t="s">
+        <v>157</v>
+      </c>
+      <c r="C33" s="56" t="s">
+        <v>27</v>
+      </c>
+      <c r="D33" s="64" t="s">
         <v>158</v>
       </c>
-      <c r="C33" s="61" t="s">
-        <v>27</v>
-      </c>
-      <c r="D33" s="70" t="s">
-        <v>159</v>
-      </c>
-      <c r="E33" s="61" t="s">
+      <c r="E33" s="56" t="s">
         <v>31</v>
       </c>
       <c r="F33" s="4"/>
@@ -2520,20 +2442,20 @@
       <c r="L33" s="50"/>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A34" s="78">
+      <c r="A34" s="69">
         <f t="shared" si="1"/>
         <v>45724</v>
       </c>
-      <c r="B34" s="67" t="s">
+      <c r="B34" s="62" t="s">
         <v>12</v>
       </c>
-      <c r="C34" s="61" t="s">
+      <c r="C34" s="56" t="s">
         <v>29</v>
       </c>
-      <c r="D34" s="70" t="s">
-        <v>130</v>
-      </c>
-      <c r="E34" s="64" t="s">
+      <c r="D34" s="64" t="s">
+        <v>129</v>
+      </c>
+      <c r="E34" s="59" t="s">
         <v>27</v>
       </c>
       <c r="F34" s="4"/>
@@ -2543,20 +2465,20 @@
       <c r="J34" s="33"/>
       <c r="K34" s="34"/>
       <c r="L34" s="50" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A35" s="78">
+      <c r="A35" s="69">
         <f t="shared" si="1"/>
         <v>45731</v>
       </c>
-      <c r="B35" s="67" t="s">
+      <c r="B35" s="62" t="s">
         <v>30</v>
       </c>
-      <c r="C35" s="61"/>
-      <c r="D35" s="72"/>
-      <c r="E35" s="63"/>
+      <c r="C35" s="56"/>
+      <c r="D35" s="66"/>
+      <c r="E35" s="58"/>
       <c r="F35" s="5"/>
       <c r="G35" s="41"/>
       <c r="H35" s="46"/>
@@ -2564,24 +2486,24 @@
       <c r="J35" s="33"/>
       <c r="K35" s="34"/>
       <c r="L35" s="50" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A36" s="78">
+      <c r="A36" s="69">
         <f t="shared" si="1"/>
         <v>45738</v>
       </c>
-      <c r="B36" s="67" t="s">
+      <c r="B36" s="62" t="s">
         <v>13</v>
       </c>
-      <c r="C36" s="61" t="s">
+      <c r="C36" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="D36" s="70" t="s">
+      <c r="D36" s="64" t="s">
         <v>25</v>
       </c>
-      <c r="E36" s="61" t="s">
+      <c r="E36" s="56" t="s">
         <v>29</v>
       </c>
       <c r="F36" s="4"/>
@@ -2594,18 +2516,18 @@
       <c r="N36" s="11"/>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A37" s="78">
+      <c r="A37" s="69">
         <f t="shared" si="1"/>
         <v>45745</v>
       </c>
-      <c r="B37" s="67" t="s">
+      <c r="B37" s="62" t="s">
         <v>128</v>
       </c>
-      <c r="C37" s="61"/>
-      <c r="D37" s="72" t="s">
+      <c r="C37" s="56"/>
+      <c r="D37" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="E37" s="61" t="s">
+      <c r="E37" s="56" t="s">
         <v>29</v>
       </c>
       <c r="F37" s="5"/>
@@ -2617,20 +2539,20 @@
       <c r="L37" s="50"/>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A38" s="78">
+      <c r="A38" s="69">
         <f>+A37+7</f>
         <v>45752</v>
       </c>
-      <c r="B38" s="67" t="s">
+      <c r="B38" s="62" t="s">
         <v>36</v>
       </c>
-      <c r="C38" s="61" t="s">
+      <c r="C38" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="D38" s="72" t="s">
+      <c r="D38" s="66" t="s">
         <v>19</v>
       </c>
-      <c r="E38" s="61" t="s">
+      <c r="E38" s="56" t="s">
         <v>29</v>
       </c>
       <c r="F38" s="5"/>
@@ -2642,18 +2564,18 @@
       <c r="L38" s="50"/>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A39" s="80">
+      <c r="A39" s="71">
         <f>+A38+7</f>
         <v>45759</v>
       </c>
-      <c r="B39" s="67" t="s">
-        <v>160</v>
-      </c>
-      <c r="C39" s="61" t="s">
+      <c r="B39" s="62" t="s">
+        <v>159</v>
+      </c>
+      <c r="C39" s="56" t="s">
         <v>31</v>
       </c>
-      <c r="D39" s="72"/>
-      <c r="E39" s="64"/>
+      <c r="D39" s="66"/>
+      <c r="E39" s="59"/>
       <c r="F39" s="5"/>
       <c r="G39" s="41"/>
       <c r="H39" s="41"/>
@@ -2663,16 +2585,16 @@
       <c r="L39" s="50"/>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A40" s="78">
-        <f t="shared" ref="A40:A44" si="2">+A39+7</f>
+      <c r="A40" s="69">
+        <f t="shared" ref="A40:A42" si="2">+A39+7</f>
         <v>45766</v>
       </c>
-      <c r="B40" s="67" t="s">
+      <c r="B40" s="62" t="s">
         <v>30</v>
       </c>
-      <c r="C40" s="61"/>
-      <c r="D40" s="70"/>
-      <c r="E40" s="61"/>
+      <c r="C40" s="56"/>
+      <c r="D40" s="64"/>
+      <c r="E40" s="56"/>
       <c r="F40" s="6"/>
       <c r="G40" s="40"/>
       <c r="H40" s="34"/>
@@ -2684,18 +2606,18 @@
       </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A41" s="78">
+      <c r="A41" s="69">
         <f t="shared" si="2"/>
         <v>45773</v>
       </c>
-      <c r="B41" s="67" t="s">
-        <v>161</v>
-      </c>
-      <c r="C41" s="61" t="s">
+      <c r="B41" s="62" t="s">
+        <v>160</v>
+      </c>
+      <c r="C41" s="56" t="s">
         <v>31</v>
       </c>
-      <c r="D41" s="72"/>
-      <c r="E41" s="61"/>
+      <c r="D41" s="66"/>
+      <c r="E41" s="56"/>
       <c r="F41" s="4"/>
       <c r="G41" s="40"/>
       <c r="H41" s="38"/>
@@ -2705,16 +2627,18 @@
       <c r="L41" s="50"/>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A42" s="78">
+      <c r="A42" s="69">
         <f t="shared" si="2"/>
         <v>45780</v>
       </c>
-      <c r="B42" s="67" t="s">
-        <v>129</v>
-      </c>
-      <c r="C42" s="61"/>
-      <c r="D42" s="72"/>
-      <c r="E42" s="61"/>
+      <c r="B42" s="62" t="s">
+        <v>161</v>
+      </c>
+      <c r="C42" s="56" t="s">
+        <v>32</v>
+      </c>
+      <c r="D42" s="66"/>
+      <c r="E42" s="56"/>
       <c r="F42" s="4"/>
       <c r="G42" s="40"/>
       <c r="H42" s="34"/>
@@ -2725,105 +2649,64 @@
       <c r="N42"/>
       <c r="O42"/>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A43" s="78">
-        <f t="shared" si="2"/>
-        <v>45787</v>
-      </c>
-      <c r="B43" s="67" t="s">
-        <v>129</v>
-      </c>
-      <c r="C43" s="61"/>
-      <c r="D43" s="72"/>
-      <c r="E43" s="61"/>
-      <c r="F43" s="4"/>
-      <c r="G43" s="40"/>
-      <c r="H43" s="34"/>
-      <c r="I43" s="38"/>
-      <c r="J43" s="33"/>
-      <c r="K43" s="34"/>
-      <c r="L43" s="50"/>
-      <c r="N43"/>
-      <c r="O43"/>
-    </row>
-    <row r="44" spans="1:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="81">
-        <f t="shared" si="2"/>
-        <v>45794</v>
-      </c>
-      <c r="B44" s="77" t="s">
-        <v>129</v>
-      </c>
-      <c r="C44" s="76"/>
-      <c r="D44" s="74"/>
-      <c r="E44" s="69"/>
-      <c r="F44" s="57"/>
-      <c r="G44" s="53"/>
-      <c r="H44" s="54"/>
-      <c r="I44" s="54"/>
-      <c r="J44" s="52"/>
-      <c r="K44" s="54"/>
-      <c r="L44" s="55"/>
-      <c r="O44"/>
-    </row>
-    <row r="45" spans="1:15" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="25"/>
-      <c r="B45" s="26" t="s">
+    <row r="43" spans="1:15" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="25"/>
+      <c r="B43" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="C45" s="13"/>
-      <c r="D45" s="27"/>
-      <c r="E45" s="28"/>
-      <c r="F45" s="29" t="s">
+      <c r="C43" s="13"/>
+      <c r="D43" s="27"/>
+      <c r="E43" s="28"/>
+      <c r="F43" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="G45" s="30"/>
-      <c r="H45" s="31"/>
-      <c r="I45" s="31"/>
-      <c r="J45" s="27"/>
-      <c r="K45" s="28"/>
-      <c r="L45" s="29"/>
+      <c r="G43" s="30"/>
+      <c r="H43" s="31"/>
+      <c r="I43" s="31"/>
+      <c r="J43" s="27"/>
+      <c r="K43" s="28"/>
+      <c r="L43" s="29"/>
+    </row>
+    <row r="44" spans="1:15" ht="19" x14ac:dyDescent="0.25">
+      <c r="A44" s="32" t="s">
+        <v>155</v>
+      </c>
+      <c r="C44" s="18"/>
+    </row>
+    <row r="45" spans="1:15" ht="21" x14ac:dyDescent="0.25">
+      <c r="A45" s="19"/>
     </row>
     <row r="46" spans="1:15" ht="19" x14ac:dyDescent="0.25">
-      <c r="A46" s="32" t="s">
-        <v>156</v>
-      </c>
-      <c r="C46" s="18"/>
-    </row>
-    <row r="47" spans="1:15" ht="21" x14ac:dyDescent="0.25">
-      <c r="A47" s="19"/>
-    </row>
-    <row r="48" spans="1:15" ht="19" x14ac:dyDescent="0.25">
-      <c r="A48" s="20" t="s">
+      <c r="A46" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="C48" s="21"/>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A88" s="15">
+      <c r="C46" s="21"/>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A86" s="15">
         <v>45171</v>
       </c>
-      <c r="B88" s="14" t="e">
-        <f>VLOOKUP(A88,Data,2,FALSE)</f>
+      <c r="B86" s="14" t="e">
+        <f>VLOOKUP(A86,Data,2,FALSE)</f>
         <v>#REF!</v>
       </c>
-      <c r="C88" s="13" t="e">
-        <f>VLOOKUP(A88,Data,3,FALSE)</f>
+      <c r="C86" s="13" t="e">
+        <f>VLOOKUP(A86,Data,3,FALSE)</f>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="114" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F114" t="s">
+    <row r="112" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F112" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="115" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F115" t="s">
+    <row r="113" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F113" t="s">
         <v>5</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:L48" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A3:L46" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:L1"/>
   </mergeCells>
@@ -3435,47 +3318,47 @@
   <sheetData>
     <row r="3" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="6" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="10" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="11" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="12" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>